<commit_message>
I completed my analysis. PPT is a WIP. Graphs and data are in excel files
</commit_message>
<xml_diff>
--- a/week-04/Market Share in vodka and rum.xlsx
+++ b/week-04/Market Share in vodka and rum.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\onurkaraer\Documents\DataAnalytics\week-04\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3EE6443-5B6E-42A5-8FD5-607A8138D9A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBEF993A-B16A-492A-91A2-90681D46D3EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{BE67EC8E-4C65-4CF7-B2D5-DECD69E644FF}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BE67EC8E-4C65-4CF7-B2D5-DECD69E644FF}"/>
   </bookViews>
   <sheets>
     <sheet name="data-1777492763550" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="12">
   <si>
     <t>vendor_group</t>
   </si>
@@ -215,7 +215,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -393,6 +393,12 @@
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.39997558519241921"/>
         <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -557,10 +563,12 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="42" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="8" fontId="0" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -618,6 +626,1842 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:pieChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'data-1777492763550'!$B$12</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>category_revenue</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-77E9-4BED-A269-30B3C64B96C7}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-77E9-4BED-A269-30B3C64B96C7}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000005-77E9-4BED-A269-30B3C64B96C7}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="3"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent4"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000007-77E9-4BED-A269-30B3C64B96C7}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="4"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent5"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000009-77E9-4BED-A269-30B3C64B96C7}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dLbls>
+            <c:spPr>
+              <a:solidFill>
+                <a:sysClr val="window" lastClr="FFFFFF"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000">
+                    <a:lumMod val="25000"/>
+                    <a:lumOff val="75000"/>
+                  </a:sysClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="dk1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="1"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="1"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:spPr xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                  <a:prstGeom prst="wedgeRectCallout">
+                    <a:avLst/>
+                  </a:prstGeom>
+                  <a:noFill/>
+                  <a:ln>
+                    <a:noFill/>
+                  </a:ln>
+                </c15:spPr>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'data-1777492763550'!$A$13:$A$17</c:f>
+              <c:strCache>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>Diageo Americas</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Bacardi</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Others</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Pernod Ricard</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Luxco</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'data-1777492763550'!$B$13:$B$17</c:f>
+              <c:numCache>
+                <c:formatCode>"$"#,##0.00_);[Red]\("$"#,##0.00\)</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>25641733.16</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>10566827.359999999</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>9036864.3599999994</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4148866.69</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>3732361.62</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-C65F-4597-A045-45831E07627E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:showLeaderLines val="0"/>
+        </c:dLbls>
+        <c:firstSliceAng val="0"/>
+      </c:pieChart>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Vodka Market Share</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:pieChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$B$11</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>category_revenue</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-CCB8-4344-A761-C4EA246F1505}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-CCB8-4344-A761-C4EA246F1505}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000005-CCB8-4344-A761-C4EA246F1505}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="3"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent4"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000007-CCB8-4344-A761-C4EA246F1505}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="4"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent5"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000009-CCB8-4344-A761-C4EA246F1505}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet1!$A$12:$A$16</c:f>
+              <c:strCache>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>Others</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Diageo Americas</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Pernod Ricard</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Luxco</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Bacardi</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$B$12:$B$16</c:f>
+              <c:numCache>
+                <c:formatCode>"$"#,##0.00_);[Red]\("$"#,##0.00\)</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>46258863.420000002</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>19082595.370000001</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>10904201.68</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>9947284.8100000005</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>6800759.8799999999</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-A4A2-4CFE-8E5D-C3F53A693A64}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:showLeaderLines val="1"/>
+        </c:dLbls>
+        <c:firstSliceAng val="0"/>
+      </c:pieChart>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="251">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="25400">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="251">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="25400">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>533400</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>52387</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>228600</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>128587</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6897B12E-200B-D8BE-2916-E45BB8F1719B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>342900</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>52387</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>128587</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E2BDE822-636E-95A8-35B2-09AA28E3F60F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -937,11 +2781,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{677E6075-2EE9-4F34-952C-A7C661EB684A}">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="16.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="24.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1040,18 +2884,67 @@
         <v>53126653.18999999</v>
       </c>
     </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>0</v>
+      </c>
+      <c r="B12" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>4</v>
+      </c>
+      <c r="B13" s="1">
+        <v>25641733.16</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B14" s="4">
+        <v>10566827.359999999</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>7</v>
+      </c>
+      <c r="B15" s="1">
+        <v>9036864.3599999994</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>8</v>
+      </c>
+      <c r="B16" s="1">
+        <v>4148866.69</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>9</v>
+      </c>
+      <c r="B17" s="1">
+        <v>3732361.62</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3CEF43B9-D155-4E8F-A7F0-108874549C04}">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="16.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -1149,7 +3042,56 @@
         <v>92993705.159999996</v>
       </c>
     </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>0</v>
+      </c>
+      <c r="B11" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>7</v>
+      </c>
+      <c r="B12" s="1">
+        <v>46258863.420000002</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>4</v>
+      </c>
+      <c r="B13" s="1">
+        <v>19082595.370000001</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>8</v>
+      </c>
+      <c r="B14" s="1">
+        <v>10904201.68</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>9</v>
+      </c>
+      <c r="B15" s="1">
+        <v>9947284.8100000005</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>6</v>
+      </c>
+      <c r="B16" s="1">
+        <v>6800759.8799999999</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Finalized my analysis and presentation. Shared video link in a txt file. Added README file with project description.
</commit_message>
<xml_diff>
--- a/week-04/Market Share in vodka and rum.xlsx
+++ b/week-04/Market Share in vodka and rum.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\onurkaraer\Documents\DataAnalytics\week-04\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBEF993A-B16A-492A-91A2-90681D46D3EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B6EF931-FEB9-4E49-9CA9-51B443F407FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BE67EC8E-4C65-4CF7-B2D5-DECD69E644FF}"/>
   </bookViews>
   <sheets>
-    <sheet name="data-1777492763550" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
+    <sheet name="rum" sheetId="1" r:id="rId1"/>
+    <sheet name="vodka" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -615,7 +615,11 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <numFmt numFmtId="12" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -652,7 +656,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>'data-1777492763550'!$B$12</c:f>
+              <c:f>rum!$B$12</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -822,7 +826,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'data-1777492763550'!$A$13:$A$17</c:f>
+              <c:f>rum!$A$13:$A$17</c:f>
               <c:strCache>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
@@ -845,7 +849,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'data-1777492763550'!$B$13:$B$17</c:f>
+              <c:f>rum!$B$13:$B$17</c:f>
               <c:numCache>
                 <c:formatCode>"$"#,##0.00_);[Red]\("$"#,##0.00\)</c:formatCode>
                 <c:ptCount val="5"/>
@@ -951,6 +955,298 @@
   </mc:AlternateContent>
   <c:chart>
     <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="bar"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>rum!$B$12</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>category_revenue</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>rum!$A$13:$A$17</c:f>
+              <c:strCache>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>Diageo Americas</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Bacardi</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Others</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Pernod Ricard</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Luxco</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>rum!$B$13:$B$17</c:f>
+              <c:numCache>
+                <c:formatCode>"$"#,##0.00_);[Red]\("$"#,##0.00\)</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>25641733.16</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>10566827.359999999</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>9036864.3599999994</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4148866.69</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>3732361.62</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-8F3C-4EA0-AC0E-989C25EAF548}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="182"/>
+        <c:axId val="2055982832"/>
+        <c:axId val="2055973232"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="2055982832"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="2055973232"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="2055973232"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="2055982832"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
       <c:tx>
         <c:rich>
           <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
@@ -1015,7 +1311,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!$B$11</c:f>
+              <c:f>vodka!$B$11</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1126,7 +1422,7 @@
           </c:dPt>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$A$12:$A$16</c:f>
+              <c:f>vodka!$A$12:$A$16</c:f>
               <c:strCache>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
@@ -1149,7 +1445,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$B$12:$B$16</c:f>
+              <c:f>vodka!$B$12:$B$16</c:f>
               <c:numCache>
                 <c:formatCode>"$"#,##0.00_);[Red]\("$"#,##0.00\)</c:formatCode>
                 <c:ptCount val="5"/>
@@ -1344,6 +1640,46 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="251">
   <cs:axisTitle>
@@ -1864,6 +2200,511 @@
 </file>
 
 <file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="216">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="251">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -2415,6 +3256,42 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>533400</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>52387</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>228600</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>128587</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FF345492-E5D9-8DFA-AA24-2F6ADCD446BE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2462,6 +3339,20 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E1A78A7A-D622-4836-91F9-4AA0E69D41B8}" name="Table1" displayName="Table1" ref="A12:B17" totalsRowShown="0">
+  <autoFilter ref="A12:B17" xr:uid="{E1A78A7A-D622-4836-91F9-4AA0E69D41B8}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A13:B17">
+    <sortCondition descending="1" ref="B12:B17"/>
+  </sortState>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{77551D96-BA85-4FDC-8EA8-DA45E1E49BCD}" name="vendor_group"/>
+    <tableColumn id="2" xr3:uid="{B0DE714C-D383-4AD6-9225-4BA3E7AA938F}" name="category_revenue" dataDxfId="0"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2785,7 +3676,8 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.140625" customWidth="1"/>
+    <col min="3" max="3" width="16.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="24.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2935,6 +3827,9 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
 </worksheet>
 </file>
 

</xml_diff>